<commit_message>
new comparison models developed to be used for accuracy comparison. readme changed.
</commit_message>
<xml_diff>
--- a/CSO_prediction/results/output_of_models.xlsx
+++ b/CSO_prediction/results/output_of_models.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofexeteruk-my.sharepoint.com/personal/mr861_exeter_ac_uk/Documents/Desktop/model_Faf/results/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofexeteruk-my.sharepoint.com/personal/mr861_exeter_ac_uk/Documents/Desktop/model_Faf/CSO_prediction/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="533" documentId="11_F25DC773A252ABDACC10484C319C55345ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E446B72-D9DF-4848-8196-A05A47F0403D}"/>
+  <xr:revisionPtr revIDLastSave="536" documentId="11_F25DC773A252ABDACC10484C319C55345ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{01D55678-56D0-40E9-8EDD-75EBD8A35BE5}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1978,4 +1978,10 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{912a5d77-fb98-4eee-af32-1334d8f04a53}" enabled="0" method="" siteId="{912a5d77-fb98-4eee-af32-1334d8f04a53}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>